<commit_message>
First part of refactoring with myLib functions
</commit_message>
<xml_diff>
--- a/data/raw/market_data2.xlsx
+++ b/data/raw/market_data2.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{7EC56965-4D77-4C9C-9B0D-FBA4994D9807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C36F348A-E20F-4296-BB96-81103D3C3C0E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2220" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{D28E9BA4-4557-4B46-B1A0-6510D1B70C36}"/>
+    <workbookView xWindow="4308" yWindow="5124" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{D28E9BA4-4557-4B46-B1A0-6510D1B70C36}"/>
   </bookViews>
   <sheets>
     <sheet name="CDS spread_2023" sheetId="1" r:id="rId1"/>
@@ -1883,12 +1883,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B04C5C0-9EBB-C64B-A016-C1201E00FA93}">
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>45042</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C2" s="6" t="s">
         <v>0</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B3" s="2">
         <v>0.5</v>
       </c>
@@ -1948,7 +1948,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -2012,7 +2012,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B6" s="4">
         <v>3</v>
       </c>
@@ -2044,7 +2044,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -2076,7 +2076,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -2108,7 +2108,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -2140,7 +2140,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B10" s="4">
         <v>10</v>
       </c>
@@ -2172,7 +2172,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>20</v>
       </c>
@@ -2204,7 +2204,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B12" s="5">
         <v>30</v>
       </c>
@@ -2236,12 +2236,12 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -2254,14 +2254,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A0CFC44-A340-4951-BAF4-0E0FCDA1C1EA}">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.19921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>45861</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="19" t="s">
         <v>0</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B3" s="2">
         <v>0.5</v>
       </c>
@@ -2313,7 +2313,7 @@
       <c r="O3" s="17"/>
       <c r="P3" s="17"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -2338,7 +2338,7 @@
       <c r="M4" s="17"/>
       <c r="N4" s="17"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -2363,7 +2363,7 @@
       <c r="M5" s="17"/>
       <c r="N5" s="17"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="4">
         <v>3</v>
       </c>
@@ -2388,7 +2388,7 @@
       <c r="M6" s="17"/>
       <c r="N6" s="17"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -2413,7 +2413,7 @@
       <c r="M7" s="17"/>
       <c r="N7" s="17"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -2438,7 +2438,7 @@
       <c r="M8" s="17"/>
       <c r="N8" s="17"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -2463,7 +2463,7 @@
       <c r="M9" s="17"/>
       <c r="N9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="4">
         <v>10</v>
       </c>
@@ -2488,7 +2488,7 @@
       <c r="M10" s="17"/>
       <c r="N10" s="17"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>20</v>
       </c>
@@ -2513,7 +2513,7 @@
       <c r="M11" s="17"/>
       <c r="N11" s="17"/>
     </row>
-    <row r="12" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="5">
         <v>30</v>
       </c>
@@ -2538,12 +2538,12 @@
       <c r="M12" s="17"/>
       <c r="N12" s="17"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -2556,18 +2556,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECE97A5D-E729-42F7-ABB8-1CDAB216BEB3}">
   <dimension ref="A1:H33"/>
-  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.75" style="9"/>
-    <col min="2" max="3" width="17.75" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.125" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.75" style="9"/>
-    <col min="7" max="7" width="21.75" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="31.625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.75" style="9"/>
+    <col min="1" max="1" width="10.69921875" style="9"/>
+    <col min="2" max="3" width="17.69921875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.09765625" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.69921875" style="9"/>
+    <col min="7" max="7" width="21.69921875" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="31.59765625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.69921875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
@@ -2578,7 +2578,7 @@
         <v>45861</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>10</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="39">
         <f>1/12</f>
         <v>8.3333333333333329E-2</v>
@@ -2621,7 +2621,7 @@
         <v>3.2327294803469395</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="13">
         <v>0.25</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>2.8540467855311089</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>0.5</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>2.6122245647754587</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="13">
         <v>0.75</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>2.465268077997838</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>1</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>2.38267356667264</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="13">
         <v>2</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>2.3428540768277779</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>3</v>
       </c>
@@ -2759,7 +2759,7 @@
         <v>2.3307797258652583</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13">
         <v>4</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>2.3360976142361105</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>5</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>2.3517320081205502</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="13">
         <v>6</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>2.3728804581851621</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>7</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>2.3963093375427924</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="13">
         <v>8</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>2.4198655535386844</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
         <v>9</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>2.4421401986570315</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="13">
         <v>10</v>
       </c>
@@ -2941,7 +2941,7 @@
         <v>2.4622373336130505</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="13">
         <v>15</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>2.4796148970621443</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="13">
         <v>20</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>2.4939749179336741</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="13">
         <v>25</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>2.5051874242513881</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>30</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>2.513237438846244</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G22" s="9">
         <v>19</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>2.5181878622416107</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E23" s="9">
         <f>SUM(E8:E21)</f>
         <v>1.0052604518849761E-2</v>
@@ -3067,7 +3067,7 @@
         <v>2.5201533514421643</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>17</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>2.51928186045286</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G25" s="9">
         <v>22</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>2.5157415581919307</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="38" t="s">
         <v>16</v>
       </c>
@@ -3103,7 +3103,7 @@
         <v>2.5097115487312003</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
         <v>15</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>2.5013752998742227</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
         <v>14</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>2.4909160141656468</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
         <v>13</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>2.4785134016524495</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
         <v>12</v>
       </c>
@@ -3163,7 +3163,7 @@
         <v>2.4643414694948689</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="38" t="s">
         <v>11</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>2.4485670521421765</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G32" s="9">
         <v>29</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>2.4313488821677161</v>
       </c>
     </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G33" s="9">
         <v>30</v>
       </c>

</xml_diff>